<commit_message>
update PCB and code
</commit_message>
<xml_diff>
--- a/adresse TCA_INA.xlsx
+++ b/adresse TCA_INA.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/electron_rare/Documents/Lelectron_rare/1-KXKM/KXKM_Batterie_Parallelator/PCB BMU v2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/electron_rare/Documents/Lelectron_rare/1-KXKM/KXKM_Batterie_Parallelator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9646D71-CADB-4F49-809A-78428AC60084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE447129-6B0C-FD43-A7ED-226EDDD3E789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{A0C7F977-36CB-0141-BBD9-870510C5852D}"/>
+    <workbookView xWindow="4340" yWindow="2820" windowWidth="25880" windowHeight="17440" xr2:uid="{A0C7F977-36CB-0141-BBD9-870510C5852D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="31">
   <si>
     <t>adresse TCA</t>
   </si>
@@ -102,6 +102,33 @@
   </si>
   <si>
     <t>0x4F</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A0</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>H</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>VCC</t>
+  </si>
+  <si>
+    <t>SDA</t>
+  </si>
+  <si>
+    <t>SCL</t>
   </si>
 </sst>
 </file>
@@ -158,12 +185,14 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -180,6 +209,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>800100</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F830567-4CA6-9756-6838-15D1C95F4F22}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7531100" y="3556000"/>
+          <a:ext cx="6972300" cy="4406900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>162560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>121920</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>88632</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3A129A7-8517-98BD-DCB9-2427BAA863FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4843780" y="2194560"/>
+          <a:ext cx="7764780" cy="5209272"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,196 +621,405 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A81A59-04D4-DF42-B4D7-8C2EB9ABD52A}">
-  <dimension ref="B1:C33"/>
+  <dimension ref="B1:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="3.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.5" customWidth="1"/>
+    <col min="8" max="8" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B2" s="3" t="s">
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B3" s="3"/>
-      <c r="C3" s="4" t="s">
+      <c r="G2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2">
+        <v>1000000</v>
+      </c>
+      <c r="K2" t="str">
+        <f>BIN2HEX(J2)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="4" t="s">
+      <c r="G3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3">
+        <v>1000001</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K5" si="0">BIN2HEX(J3)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
-      <c r="C5" s="4" t="s">
+      <c r="G4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4">
+        <v>1000010</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B6" s="3" t="s">
+      <c r="G5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5">
+        <v>1000011</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B7" s="3"/>
-      <c r="C7" s="4" t="s">
+      <c r="G6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B8" s="3"/>
-      <c r="C8" s="4" t="s">
+      <c r="G7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B9" s="3"/>
-      <c r="C9" s="4" t="s">
+      <c r="G8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B10" s="3" t="s">
+      <c r="G9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B11" s="3"/>
-      <c r="C11" s="4" t="s">
+      <c r="G10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B12" s="3"/>
-      <c r="C12" s="4" t="s">
+      <c r="G11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B13" s="3"/>
-      <c r="C13" s="4" t="s">
+      <c r="G12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B14" s="3" t="s">
+      <c r="G13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B14" s="4" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="3"/>
-      <c r="C15" s="4" t="s">
+      <c r="G14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B16" s="3"/>
-      <c r="C16" s="4" t="s">
+      <c r="G15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B17" s="3"/>
-      <c r="C17" s="4" t="s">
+      <c r="G16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="2"/>
-      <c r="C18" s="1"/>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B19" s="2"/>
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B20" s="2"/>
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B21" s="2"/>
-      <c r="C21" s="1"/>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B22" s="2"/>
-      <c r="C22" s="1"/>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B23" s="2"/>
-      <c r="C23" s="1"/>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B24" s="2"/>
-      <c r="C24" s="1"/>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B25" s="2"/>
-      <c r="C25" s="1"/>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B26" s="2"/>
-      <c r="C26" s="1"/>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B27" s="2"/>
-      <c r="C27" s="1"/>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B28" s="2"/>
-      <c r="C28" s="1"/>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B29" s="2"/>
-      <c r="C29" s="1"/>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B30" s="2"/>
-      <c r="C30" s="1"/>
-    </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B31" s="2"/>
-      <c r="C31" s="1"/>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B32" s="2"/>
-      <c r="C32" s="1"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B33" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F31" s="1"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="F32" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="16">
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="E14:E17"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="B14:B17"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D10:D13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>